<commit_message>
Fixed the benchamrk to include more metrics
</commit_message>
<xml_diff>
--- a/benchmarks/benchmark_results/fcp_inference_results.xlsx
+++ b/benchmarks/benchmark_results/fcp_inference_results.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F_dimension_frequency" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C_pole_consistency" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P_subgroup_prg" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="diagnostics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,23 +420,23 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>dim</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="n">
+      <c r="B1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>age</t>
         </is>
@@ -463,7 +452,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>education</t>
         </is>
@@ -479,7 +468,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
@@ -495,7 +484,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>orientation</t>
         </is>
@@ -511,7 +500,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>politics</t>
         </is>
@@ -541,29 +530,29 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>subgroup</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>n_s</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>frac_toxic</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>frac_civil</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>(('education', 'low'),)</t>
         </is>
@@ -579,7 +568,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>(('education', 'high'),)</t>
         </is>
@@ -595,7 +584,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'),)</t>
         </is>
@@ -611,7 +600,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'),)</t>
         </is>
@@ -627,7 +616,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>(('education', 'medium'),)</t>
         </is>
@@ -643,7 +632,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>(('politics', 'center'),)</t>
         </is>
@@ -659,7 +648,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>(('politics', 'left'),)</t>
         </is>
@@ -675,7 +664,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>(('politics', 'right'),)</t>
         </is>
@@ -691,7 +680,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'))</t>
         </is>
@@ -707,7 +696,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('politics', 'center'))</t>
         </is>
@@ -723,7 +712,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'female'))</t>
         </is>
@@ -739,7 +728,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'))</t>
         </is>
@@ -755,7 +744,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -771,7 +760,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'),)</t>
         </is>
@@ -787,7 +776,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'))</t>
         </is>
@@ -803,7 +792,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -819,7 +808,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -835,7 +824,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'))</t>
         </is>
@@ -851,7 +840,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -867,7 +856,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -883,7 +872,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>(('gender', 'female'),)</t>
         </is>
@@ -899,7 +888,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -915,7 +904,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'))</t>
         </is>
@@ -931,7 +920,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'),)</t>
         </is>
@@ -947,7 +936,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'),)</t>
         </is>
@@ -963,7 +952,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'))</t>
         </is>
@@ -979,7 +968,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -995,7 +984,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'))</t>
         </is>
@@ -1011,7 +1000,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>(('age', '25-50'),)</t>
         </is>
@@ -1027,7 +1016,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'))</t>
         </is>
@@ -1043,7 +1032,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1059,7 +1048,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('politics', 'right'))</t>
         </is>
@@ -1075,7 +1064,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -1091,7 +1080,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'non-binary'))</t>
         </is>
@@ -1107,7 +1096,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'))</t>
         </is>
@@ -1123,7 +1112,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -1139,7 +1128,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1155,7 +1144,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -1171,7 +1160,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1187,7 +1176,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('politics', 'left'))</t>
         </is>
@@ -1203,7 +1192,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1219,7 +1208,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -1235,7 +1224,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>(('gender', 'male'),)</t>
         </is>
@@ -1251,7 +1240,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -1267,7 +1256,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -1283,7 +1272,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -1299,7 +1288,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1315,7 +1304,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('politics', 'left'))</t>
         </is>
@@ -1331,7 +1320,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('politics', 'right'))</t>
         </is>
@@ -1347,7 +1336,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1363,7 +1352,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1379,7 +1368,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1395,7 +1384,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1411,7 +1400,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1427,7 +1416,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1443,7 +1432,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1459,7 +1448,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'))</t>
         </is>
@@ -1475,7 +1464,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -1491,7 +1480,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1507,7 +1496,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -1523,7 +1512,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -1539,7 +1528,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'))</t>
         </is>
@@ -1555,7 +1544,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1571,7 +1560,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -1587,7 +1576,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -1603,7 +1592,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -1619,7 +1608,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -1635,7 +1624,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1651,7 +1640,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1667,7 +1656,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1683,7 +1672,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1699,7 +1688,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'))</t>
         </is>
@@ -1715,7 +1704,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -1731,7 +1720,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('politics', 'center'))</t>
         </is>
@@ -1747,7 +1736,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1763,7 +1752,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -1779,7 +1768,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'))</t>
         </is>
@@ -1795,7 +1784,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1811,7 +1800,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -1827,7 +1816,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -1843,7 +1832,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -1859,7 +1848,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="inlineStr">
+      <c r="A83" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -1875,7 +1864,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1891,7 +1880,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="inlineStr">
+      <c r="A85" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1907,7 +1896,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="inlineStr">
+      <c r="A86" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1923,7 +1912,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="inlineStr">
+      <c r="A87" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1939,7 +1928,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="inlineStr">
+      <c r="A88" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -1955,7 +1944,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="inlineStr">
+      <c r="A89" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -1971,7 +1960,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="inlineStr">
+      <c r="A90" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -1987,7 +1976,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="inlineStr">
+      <c r="A91" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -2003,7 +1992,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="inlineStr">
+      <c r="A92" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -2019,7 +2008,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="inlineStr">
+      <c r="A93" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -2035,7 +2024,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="inlineStr">
+      <c r="A94" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'))</t>
         </is>
@@ -2051,7 +2040,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="inlineStr">
+      <c r="A95" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('politics', 'right'))</t>
         </is>
@@ -2067,7 +2056,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="inlineStr">
+      <c r="A96" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -2083,7 +2072,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="inlineStr">
+      <c r="A97" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2099,7 +2088,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2115,7 +2104,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="inlineStr">
+      <c r="A99" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2131,7 +2120,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="inlineStr">
+      <c r="A100" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2147,7 +2136,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="inlineStr">
+      <c r="A101" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2163,7 +2152,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="inlineStr">
+      <c r="A102" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2179,7 +2168,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="inlineStr">
+      <c r="A103" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2195,7 +2184,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="inlineStr">
+      <c r="A104" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -2211,7 +2200,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="inlineStr">
+      <c r="A105" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2227,7 +2216,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="inlineStr">
+      <c r="A106" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'))</t>
         </is>
@@ -2243,7 +2232,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="inlineStr">
+      <c r="A107" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2259,7 +2248,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="inlineStr">
+      <c r="A108" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('politics', 'right'))</t>
         </is>
@@ -2275,7 +2264,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="inlineStr">
+      <c r="A109" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2291,7 +2280,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="inlineStr">
+      <c r="A110" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2307,7 +2296,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="inlineStr">
+      <c r="A111" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'))</t>
         </is>
@@ -2323,7 +2312,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="inlineStr">
+      <c r="A112" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -2339,7 +2328,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="inlineStr">
+      <c r="A113" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -2355,7 +2344,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="inlineStr">
+      <c r="A114" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -2371,7 +2360,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="inlineStr">
+      <c r="A115" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -2387,7 +2376,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="inlineStr">
+      <c r="A116" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2403,7 +2392,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="inlineStr">
+      <c r="A117" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('politics', 'center'))</t>
         </is>
@@ -2419,7 +2408,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="inlineStr">
+      <c r="A118" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -2435,7 +2424,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="inlineStr">
+      <c r="A119" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -2451,7 +2440,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="inlineStr">
+      <c r="A120" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('politics', 'center'))</t>
         </is>
@@ -2467,7 +2456,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="inlineStr">
+      <c r="A121" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('gender', 'female'))</t>
         </is>
@@ -2483,7 +2472,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="inlineStr">
+      <c r="A122" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('politics', 'right'))</t>
         </is>
@@ -2499,7 +2488,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="inlineStr">
+      <c r="A123" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'))</t>
         </is>
@@ -2515,7 +2504,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="inlineStr">
+      <c r="A124" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2531,7 +2520,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="inlineStr">
+      <c r="A125" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -2547,7 +2536,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="inlineStr">
+      <c r="A126" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2563,7 +2552,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="inlineStr">
+      <c r="A127" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2579,7 +2568,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="inlineStr">
+      <c r="A128" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -2595,7 +2584,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="inlineStr">
+      <c r="A129" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -2611,7 +2600,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="inlineStr">
+      <c r="A130" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -2627,7 +2616,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="inlineStr">
+      <c r="A131" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -2643,7 +2632,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="inlineStr">
+      <c r="A132" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -2659,7 +2648,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="inlineStr">
+      <c r="A133" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -2675,7 +2664,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="inlineStr">
+      <c r="A134" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -2691,7 +2680,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="inlineStr">
+      <c r="A135" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -2707,7 +2696,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="inlineStr">
+      <c r="A136" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -2723,7 +2712,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="inlineStr">
+      <c r="A137" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('politics', 'center'))</t>
         </is>
@@ -2739,7 +2728,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="inlineStr">
+      <c r="A138" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -2755,7 +2744,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="inlineStr">
+      <c r="A139" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -2771,7 +2760,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="inlineStr">
+      <c r="A140" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -2787,7 +2776,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="inlineStr">
+      <c r="A141" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -2803,7 +2792,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="inlineStr">
+      <c r="A142" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('politics', 'right'))</t>
         </is>
@@ -2819,7 +2808,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="inlineStr">
+      <c r="A143" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -2835,7 +2824,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2851,7 +2840,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="inlineStr">
+      <c r="A145" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -2867,7 +2856,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="inlineStr">
+      <c r="A146" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -2883,7 +2872,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="inlineStr">
+      <c r="A147" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -2899,7 +2888,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2915,7 +2904,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="inlineStr">
+      <c r="A149" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -2931,7 +2920,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="inlineStr">
+      <c r="A150" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -2947,7 +2936,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="inlineStr">
+      <c r="A151" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -2963,7 +2952,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="inlineStr">
+      <c r="A152" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -2979,7 +2968,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="inlineStr">
+      <c r="A153" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -2995,7 +2984,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="inlineStr">
+      <c r="A154" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3011,7 +3000,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="inlineStr">
+      <c r="A155" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'))</t>
         </is>
@@ -3027,7 +3016,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="inlineStr">
+      <c r="A156" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -3043,7 +3032,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="inlineStr">
+      <c r="A157" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -3059,7 +3048,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="inlineStr">
+      <c r="A158" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3075,7 +3064,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="inlineStr">
+      <c r="A159" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -3091,7 +3080,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="inlineStr">
+      <c r="A160" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'))</t>
         </is>
@@ -3107,7 +3096,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="inlineStr">
+      <c r="A161" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -3123,7 +3112,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="inlineStr">
+      <c r="A162" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -3139,7 +3128,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="inlineStr">
+      <c r="A163" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('politics', 'center'))</t>
         </is>
@@ -3155,7 +3144,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="inlineStr">
+      <c r="A164" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -3171,7 +3160,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="inlineStr">
+      <c r="A165" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -3187,7 +3176,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="inlineStr">
+      <c r="A166" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -3203,7 +3192,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="inlineStr">
+      <c r="A167" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -3219,7 +3208,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="inlineStr">
+      <c r="A168" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -3235,7 +3224,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="inlineStr">
+      <c r="A169" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -3251,7 +3240,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="inlineStr">
+      <c r="A170" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('politics', 'right'))</t>
         </is>
@@ -3267,7 +3256,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="inlineStr">
+      <c r="A171" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -3283,7 +3272,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="inlineStr">
+      <c r="A172" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3299,7 +3288,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="inlineStr">
+      <c r="A173" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('gender', 'male'))</t>
         </is>
@@ -3315,7 +3304,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="inlineStr">
+      <c r="A174" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -3331,7 +3320,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="inlineStr">
+      <c r="A175" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -3347,7 +3336,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="inlineStr">
+      <c r="A176" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -3363,7 +3352,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="inlineStr">
+      <c r="A177" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3379,7 +3368,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="inlineStr">
+      <c r="A178" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -3395,7 +3384,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="inlineStr">
+      <c r="A179" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('politics', 'left'))</t>
         </is>
@@ -3411,7 +3400,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="inlineStr">
+      <c r="A180" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -3427,7 +3416,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="inlineStr">
+      <c r="A181" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('gender', 'non-binary'))</t>
         </is>
@@ -3443,7 +3432,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="inlineStr">
+      <c r="A182" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3459,7 +3448,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="inlineStr">
+      <c r="A183" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -3475,7 +3464,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="inlineStr">
+      <c r="A184" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -3491,7 +3480,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="inlineStr">
+      <c r="A185" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('gender', 'female'))</t>
         </is>
@@ -3507,7 +3496,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="inlineStr">
+      <c r="A186" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'), ('politics', 'left'))</t>
         </is>
@@ -3523,7 +3512,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="inlineStr">
+      <c r="A187" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('gender', 'non-binary'))</t>
         </is>
@@ -3539,7 +3528,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="inlineStr">
+      <c r="A188" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('gender', 'male'))</t>
         </is>
@@ -3555,7 +3544,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="inlineStr">
+      <c r="A189" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3571,7 +3560,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="inlineStr">
+      <c r="A190" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('politics', 'center'))</t>
         </is>
@@ -3587,7 +3576,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="inlineStr">
+      <c r="A191" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -3603,7 +3592,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="inlineStr">
+      <c r="A192" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('politics', 'right'))</t>
         </is>
@@ -3619,7 +3608,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="inlineStr">
+      <c r="A193" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -3635,7 +3624,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="inlineStr">
+      <c r="A194" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -3651,7 +3640,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="inlineStr">
+      <c r="A195" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -3667,7 +3656,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="inlineStr">
+      <c r="A196" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -3683,7 +3672,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="inlineStr">
+      <c r="A197" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('gender', 'male'))</t>
         </is>
@@ -3699,7 +3688,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="inlineStr">
+      <c r="A198" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -3715,7 +3704,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="inlineStr">
+      <c r="A199" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('gender', 'female'))</t>
         </is>
@@ -3731,7 +3720,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="inlineStr">
+      <c r="A200" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('gender', 'non-binary'))</t>
         </is>
@@ -3747,7 +3736,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="inlineStr">
+      <c r="A201" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('politics', 'right'))</t>
         </is>
@@ -3763,7 +3752,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="inlineStr">
+      <c r="A202" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('politics', 'left'))</t>
         </is>
@@ -3779,7 +3768,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="inlineStr">
+      <c r="A203" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('politics', 'center'))</t>
         </is>
@@ -3795,7 +3784,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="inlineStr">
+      <c r="A204" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3811,7 +3800,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="inlineStr">
+      <c r="A205" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -3827,7 +3816,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="inlineStr">
+      <c r="A206" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -3843,7 +3832,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="inlineStr">
+      <c r="A207" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'))</t>
         </is>
@@ -3859,7 +3848,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="inlineStr">
+      <c r="A208" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('gender', 'female'))</t>
         </is>
@@ -3875,7 +3864,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="inlineStr">
+      <c r="A209" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -3891,7 +3880,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="inlineStr">
+      <c r="A210" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -3907,7 +3896,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="inlineStr">
+      <c r="A211" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -3923,7 +3912,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="inlineStr">
+      <c r="A212" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -3939,7 +3928,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="inlineStr">
+      <c r="A213" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -3955,7 +3944,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="inlineStr">
+      <c r="A214" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -3971,7 +3960,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="inlineStr">
+      <c r="A215" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('gender', 'non-binary'))</t>
         </is>
@@ -3987,7 +3976,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="inlineStr">
+      <c r="A216" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -4003,7 +3992,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="inlineStr">
+      <c r="A217" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('politics', 'right'))</t>
         </is>
@@ -4019,7 +4008,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="inlineStr">
+      <c r="A218" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('politics', 'center'))</t>
         </is>
@@ -4035,7 +4024,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="inlineStr">
+      <c r="A219" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('gender', 'non-binary'))</t>
         </is>
@@ -4051,7 +4040,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="inlineStr">
+      <c r="A220" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -4067,7 +4056,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="inlineStr">
+      <c r="A221" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -4083,7 +4072,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="inlineStr">
+      <c r="A222" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -4099,7 +4088,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="inlineStr">
+      <c r="A223" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -4115,7 +4104,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="inlineStr">
+      <c r="A224" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -4131,7 +4120,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="inlineStr">
+      <c r="A225" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -4147,7 +4136,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="inlineStr">
+      <c r="A226" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -4163,7 +4152,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="inlineStr">
+      <c r="A227" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -4179,7 +4168,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="inlineStr">
+      <c r="A228" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('politics', 'left'))</t>
         </is>
@@ -4195,7 +4184,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="inlineStr">
+      <c r="A229" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -4211,7 +4200,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="inlineStr">
+      <c r="A230" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -4227,7 +4216,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="inlineStr">
+      <c r="A231" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -4243,7 +4232,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="inlineStr">
+      <c r="A232" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -4259,7 +4248,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="inlineStr">
+      <c r="A233" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -4275,7 +4264,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="inlineStr">
+      <c r="A234" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'))</t>
         </is>
@@ -4291,7 +4280,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="inlineStr">
+      <c r="A235" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -4307,7 +4296,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="inlineStr">
+      <c r="A236" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -4323,7 +4312,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="inlineStr">
+      <c r="A237" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -4339,7 +4328,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="inlineStr">
+      <c r="A238" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'))</t>
         </is>
@@ -4355,7 +4344,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="inlineStr">
+      <c r="A239" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -4371,7 +4360,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="inlineStr">
+      <c r="A240" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -4387,7 +4376,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="inlineStr">
+      <c r="A241" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -4403,7 +4392,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="inlineStr">
+      <c r="A242" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('politics', 'center'))</t>
         </is>
@@ -4419,7 +4408,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="inlineStr">
+      <c r="A243" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -4435,7 +4424,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="inlineStr">
+      <c r="A244" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'))</t>
         </is>
@@ -4451,7 +4440,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="inlineStr">
+      <c r="A245" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -4467,7 +4456,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="inlineStr">
+      <c r="A246" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -4483,7 +4472,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="inlineStr">
+      <c r="A247" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -4499,7 +4488,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="1" t="inlineStr">
+      <c r="A248" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -4515,7 +4504,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="1" t="inlineStr">
+      <c r="A249" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -4531,7 +4520,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="1" t="inlineStr">
+      <c r="A250" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -4547,7 +4536,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="1" t="inlineStr">
+      <c r="A251" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -4563,7 +4552,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="1" t="inlineStr">
+      <c r="A252" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -4579,7 +4568,7 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="1" t="inlineStr">
+      <c r="A253" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -4595,7 +4584,7 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="1" t="inlineStr">
+      <c r="A254" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -4611,7 +4600,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="1" t="inlineStr">
+      <c r="A255" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -4627,7 +4616,7 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="1" t="inlineStr">
+      <c r="A256" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -4657,24 +4646,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>subgroup</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>n_s</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_prg</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -4687,7 +4676,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -4700,7 +4689,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'),)</t>
         </is>
@@ -4713,7 +4702,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'),)</t>
         </is>
@@ -4726,7 +4715,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -4739,7 +4728,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -4752,7 +4741,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -4765,7 +4754,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -4778,7 +4767,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -4791,7 +4780,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -4804,7 +4793,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -4817,7 +4806,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -4830,7 +4819,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -4843,7 +4832,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('politics', 'center'))</t>
         </is>
@@ -4856,7 +4845,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('politics', 'center'))</t>
         </is>
@@ -4869,7 +4858,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -4882,7 +4871,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -4895,7 +4884,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -4908,7 +4897,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('politics', 'right'))</t>
         </is>
@@ -4921,7 +4910,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('politics', 'right'))</t>
         </is>
@@ -4934,7 +4923,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -4947,7 +4936,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -4960,7 +4949,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -4973,7 +4962,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -4986,7 +4975,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -4999,7 +4988,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5012,7 +5001,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5025,7 +5014,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -5038,7 +5027,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5051,7 +5040,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5064,7 +5053,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>(('gender', 'male'),)</t>
         </is>
@@ -5077,7 +5066,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5090,7 +5079,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5103,7 +5092,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -5116,7 +5105,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -5129,7 +5118,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -5142,7 +5131,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -5155,7 +5144,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5168,7 +5157,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -5181,7 +5170,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -5194,7 +5183,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5207,7 +5196,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5220,7 +5209,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -5233,7 +5222,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -5246,7 +5235,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -5259,7 +5248,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5272,7 +5261,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5285,7 +5274,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -5298,7 +5287,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'),)</t>
         </is>
@@ -5311,7 +5300,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -5324,7 +5313,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>(('education', 'low'),)</t>
         </is>
@@ -5337,7 +5326,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5350,7 +5339,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>(('education', 'high'),)</t>
         </is>
@@ -5363,7 +5352,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>(('politics', 'left'),)</t>
         </is>
@@ -5376,7 +5365,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>(('politics', 'center'),)</t>
         </is>
@@ -5389,7 +5378,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'),)</t>
         </is>
@@ -5402,7 +5391,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -5415,7 +5404,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5428,7 +5417,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>(('education', 'medium'),)</t>
         </is>
@@ -5441,7 +5430,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>(('age', '25-50'),)</t>
         </is>
@@ -5454,7 +5443,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5467,7 +5456,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5480,7 +5469,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -5493,7 +5482,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5506,7 +5495,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5519,7 +5508,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5532,7 +5521,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>(('politics', 'right'),)</t>
         </is>
@@ -5545,7 +5534,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5558,7 +5547,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>(('gender', 'female'),)</t>
         </is>
@@ -5571,7 +5560,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5584,7 +5573,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -5597,7 +5586,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -5610,7 +5599,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5623,7 +5612,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -5636,7 +5625,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5649,7 +5638,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -5662,7 +5651,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -5675,7 +5664,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -5688,7 +5677,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'),)</t>
         </is>
@@ -5701,7 +5690,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -5714,7 +5703,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -5727,7 +5716,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="inlineStr">
+      <c r="A83" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -5740,7 +5729,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5753,7 +5742,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="inlineStr">
+      <c r="A85" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -5766,7 +5755,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="inlineStr">
+      <c r="A86" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -5779,7 +5768,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="inlineStr">
+      <c r="A87" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -5792,7 +5781,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="inlineStr">
+      <c r="A88" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -5805,7 +5794,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="inlineStr">
+      <c r="A89" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5818,7 +5807,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="inlineStr">
+      <c r="A90" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -5831,7 +5820,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="inlineStr">
+      <c r="A91" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -5844,7 +5833,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="inlineStr">
+      <c r="A92" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -5857,7 +5846,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="inlineStr">
+      <c r="A93" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('politics', 'center'))</t>
         </is>
@@ -5870,7 +5859,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="inlineStr">
+      <c r="A94" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -5883,7 +5872,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="inlineStr">
+      <c r="A95" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -5896,7 +5885,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="inlineStr">
+      <c r="A96" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -5909,7 +5898,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="inlineStr">
+      <c r="A97" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -5922,7 +5911,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -5935,7 +5924,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="inlineStr">
+      <c r="A99" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('politics', 'right'))</t>
         </is>
@@ -5948,7 +5937,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="inlineStr">
+      <c r="A100" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5961,7 +5950,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="inlineStr">
+      <c r="A101" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -5974,7 +5963,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="inlineStr">
+      <c r="A102" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -5987,7 +5976,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="inlineStr">
+      <c r="A103" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6000,7 +5989,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="inlineStr">
+      <c r="A104" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -6013,7 +6002,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="inlineStr">
+      <c r="A105" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -6026,7 +6015,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="inlineStr">
+      <c r="A106" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -6039,7 +6028,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="inlineStr">
+      <c r="A107" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6052,7 +6041,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="inlineStr">
+      <c r="A108" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -6065,7 +6054,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="inlineStr">
+      <c r="A109" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -6078,7 +6067,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="inlineStr">
+      <c r="A110" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -6091,7 +6080,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="inlineStr">
+      <c r="A111" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6104,7 +6093,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="inlineStr">
+      <c r="A112" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -6117,7 +6106,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="inlineStr">
+      <c r="A113" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -6130,7 +6119,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="inlineStr">
+      <c r="A114" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6143,7 +6132,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="inlineStr">
+      <c r="A115" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6156,7 +6145,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="inlineStr">
+      <c r="A116" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -6169,7 +6158,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="inlineStr">
+      <c r="A117" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -6182,7 +6171,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="inlineStr">
+      <c r="A118" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6195,7 +6184,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="inlineStr">
+      <c r="A119" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -6208,7 +6197,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="inlineStr">
+      <c r="A120" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -6221,7 +6210,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="inlineStr">
+      <c r="A121" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -6234,7 +6223,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="inlineStr">
+      <c r="A122" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -6247,7 +6236,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="inlineStr">
+      <c r="A123" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6260,7 +6249,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="inlineStr">
+      <c r="A124" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6273,7 +6262,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="inlineStr">
+      <c r="A125" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'high'))</t>
         </is>
@@ -6286,7 +6275,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="inlineStr">
+      <c r="A126" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('gender', 'male'))</t>
         </is>
@@ -6299,7 +6288,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="inlineStr">
+      <c r="A127" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('gender', 'non-binary'))</t>
         </is>
@@ -6312,7 +6301,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="inlineStr">
+      <c r="A128" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -6325,7 +6314,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="inlineStr">
+      <c r="A129" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6338,7 +6327,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="inlineStr">
+      <c r="A130" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6351,7 +6340,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="inlineStr">
+      <c r="A131" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -6364,7 +6353,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="inlineStr">
+      <c r="A132" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -6377,7 +6366,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="inlineStr">
+      <c r="A133" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -6390,7 +6379,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="inlineStr">
+      <c r="A134" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -6403,7 +6392,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="inlineStr">
+      <c r="A135" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -6416,7 +6405,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="inlineStr">
+      <c r="A136" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -6429,7 +6418,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="inlineStr">
+      <c r="A137" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -6442,7 +6431,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="inlineStr">
+      <c r="A138" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6455,7 +6444,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="inlineStr">
+      <c r="A139" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'), ('politics', 'left'))</t>
         </is>
@@ -6468,7 +6457,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="inlineStr">
+      <c r="A140" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -6481,7 +6470,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="inlineStr">
+      <c r="A141" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -6494,7 +6483,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="inlineStr">
+      <c r="A142" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -6507,7 +6496,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="inlineStr">
+      <c r="A143" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -6520,7 +6509,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -6533,7 +6522,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="inlineStr">
+      <c r="A145" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -6546,7 +6535,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="inlineStr">
+      <c r="A146" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'))</t>
         </is>
@@ -6559,7 +6548,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="inlineStr">
+      <c r="A147" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('politics', 'left'))</t>
         </is>
@@ -6572,7 +6561,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'))</t>
         </is>
@@ -6585,7 +6574,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="inlineStr">
+      <c r="A149" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'), ('politics', 'left'))</t>
         </is>
@@ -6598,7 +6587,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="inlineStr">
+      <c r="A150" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6611,7 +6600,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="inlineStr">
+      <c r="A151" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -6624,7 +6613,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="inlineStr">
+      <c r="A152" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -6637,7 +6626,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="inlineStr">
+      <c r="A153" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -6650,7 +6639,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="inlineStr">
+      <c r="A154" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('gender', 'male'))</t>
         </is>
@@ -6663,7 +6652,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="inlineStr">
+      <c r="A155" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('politics', 'right'))</t>
         </is>
@@ -6676,7 +6665,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="inlineStr">
+      <c r="A156" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('gender', 'non-binary'))</t>
         </is>
@@ -6689,7 +6678,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="inlineStr">
+      <c r="A157" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'))</t>
         </is>
@@ -6702,7 +6691,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="inlineStr">
+      <c r="A158" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'non-binary'))</t>
         </is>
@@ -6715,7 +6704,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="inlineStr">
+      <c r="A159" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('politics', 'left'))</t>
         </is>
@@ -6728,7 +6717,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="inlineStr">
+      <c r="A160" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -6741,7 +6730,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="inlineStr">
+      <c r="A161" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -6754,7 +6743,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="inlineStr">
+      <c r="A162" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'), ('gender', 'non-binary'))</t>
         </is>
@@ -6767,7 +6756,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="inlineStr">
+      <c r="A163" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'), ('gender', 'non-binary'))</t>
         </is>
@@ -6780,7 +6769,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="inlineStr">
+      <c r="A164" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('politics', 'left'))</t>
         </is>
@@ -6793,7 +6782,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="inlineStr">
+      <c r="A165" t="inlineStr">
         <is>
           <t>(('orientation', 'heterosexual'), ('politics', 'right'))</t>
         </is>
@@ -6806,7 +6795,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="inlineStr">
+      <c r="A166" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'))</t>
         </is>
@@ -6819,7 +6808,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="inlineStr">
+      <c r="A167" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('gender', 'female'))</t>
         </is>
@@ -6832,7 +6821,7 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="inlineStr">
+      <c r="A168" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -6845,7 +6834,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="inlineStr">
+      <c r="A169" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -6858,7 +6847,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="inlineStr">
+      <c r="A170" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'female'))</t>
         </is>
@@ -6871,7 +6860,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="inlineStr">
+      <c r="A171" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('politics', 'right'))</t>
         </is>
@@ -6884,7 +6873,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="inlineStr">
+      <c r="A172" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'), ('politics', 'left'))</t>
         </is>
@@ -6897,7 +6886,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="inlineStr">
+      <c r="A173" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -6910,7 +6899,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="inlineStr">
+      <c r="A174" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -6923,7 +6912,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="inlineStr">
+      <c r="A175" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'non-binary'), ('politics', 'right'))</t>
         </is>
@@ -6936,7 +6925,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="inlineStr">
+      <c r="A176" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('politics', 'right'))</t>
         </is>
@@ -6949,7 +6938,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="inlineStr">
+      <c r="A177" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('politics', 'right'))</t>
         </is>
@@ -6962,7 +6951,7 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="inlineStr">
+      <c r="A178" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('politics', 'right'))</t>
         </is>
@@ -6975,7 +6964,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="inlineStr">
+      <c r="A179" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'))</t>
         </is>
@@ -6988,7 +6977,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="inlineStr">
+      <c r="A180" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7001,7 +6990,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="inlineStr">
+      <c r="A181" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7014,7 +7003,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="inlineStr">
+      <c r="A182" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -7027,7 +7016,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="inlineStr">
+      <c r="A183" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -7040,7 +7029,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="inlineStr">
+      <c r="A184" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('politics', 'right'))</t>
         </is>
@@ -7053,7 +7042,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="inlineStr">
+      <c r="A185" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'low'))</t>
         </is>
@@ -7066,7 +7055,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="inlineStr">
+      <c r="A186" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('politics', 'center'))</t>
         </is>
@@ -7079,7 +7068,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="inlineStr">
+      <c r="A187" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'female'))</t>
         </is>
@@ -7092,7 +7081,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="inlineStr">
+      <c r="A188" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'))</t>
         </is>
@@ -7105,7 +7094,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="inlineStr">
+      <c r="A189" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'male'))</t>
         </is>
@@ -7118,7 +7107,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="inlineStr">
+      <c r="A190" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'high'))</t>
         </is>
@@ -7131,7 +7120,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="inlineStr">
+      <c r="A191" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('politics', 'center'))</t>
         </is>
@@ -7144,7 +7133,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="inlineStr">
+      <c r="A192" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7157,7 +7146,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="inlineStr">
+      <c r="A193" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'non-binary'))</t>
         </is>
@@ -7170,7 +7159,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="inlineStr">
+      <c r="A194" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'non-binary'))</t>
         </is>
@@ -7183,7 +7172,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="inlineStr">
+      <c r="A195" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'male'))</t>
         </is>
@@ -7196,7 +7185,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="inlineStr">
+      <c r="A196" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -7209,7 +7198,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="inlineStr">
+      <c r="A197" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('politics', 'center'))</t>
         </is>
@@ -7222,7 +7211,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="inlineStr">
+      <c r="A198" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7235,7 +7224,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="inlineStr">
+      <c r="A199" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'high'))</t>
         </is>
@@ -7248,7 +7237,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="inlineStr">
+      <c r="A200" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('gender', 'female'))</t>
         </is>
@@ -7261,7 +7250,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="inlineStr">
+      <c r="A201" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7274,7 +7263,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="inlineStr">
+      <c r="A202" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7287,7 +7276,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="inlineStr">
+      <c r="A203" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'))</t>
         </is>
@@ -7300,7 +7289,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="inlineStr">
+      <c r="A204" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'low'))</t>
         </is>
@@ -7313,7 +7302,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="inlineStr">
+      <c r="A205" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('politics', 'center'))</t>
         </is>
@@ -7326,7 +7315,7 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="inlineStr">
+      <c r="A206" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('education', 'medium'))</t>
         </is>
@@ -7339,7 +7328,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="inlineStr">
+      <c r="A207" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('gender', 'female'))</t>
         </is>
@@ -7352,7 +7341,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="inlineStr">
+      <c r="A208" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7365,7 +7354,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="inlineStr">
+      <c r="A209" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7378,7 +7367,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="inlineStr">
+      <c r="A210" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7391,7 +7380,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="inlineStr">
+      <c r="A211" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('politics', 'center'))</t>
         </is>
@@ -7404,7 +7393,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="1" t="inlineStr">
+      <c r="A212" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7417,7 +7406,7 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="1" t="inlineStr">
+      <c r="A213" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('politics', 'right'))</t>
         </is>
@@ -7430,7 +7419,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="1" t="inlineStr">
+      <c r="A214" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('politics', 'left'))</t>
         </is>
@@ -7443,7 +7432,7 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="1" t="inlineStr">
+      <c r="A215" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('politics', 'center'))</t>
         </is>
@@ -7456,7 +7445,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="1" t="inlineStr">
+      <c r="A216" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7469,7 +7458,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="1" t="inlineStr">
+      <c r="A217" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -7482,7 +7471,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="1" t="inlineStr">
+      <c r="A218" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'male'))</t>
         </is>
@@ -7495,7 +7484,7 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="1" t="inlineStr">
+      <c r="A219" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7508,7 +7497,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="1" t="inlineStr">
+      <c r="A220" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'non-binary'))</t>
         </is>
@@ -7521,7 +7510,7 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="1" t="inlineStr">
+      <c r="A221" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('gender', 'non-binary'), ('politics', 'left'))</t>
         </is>
@@ -7534,7 +7523,7 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="1" t="inlineStr">
+      <c r="A222" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('politics', 'center'))</t>
         </is>
@@ -7547,7 +7536,7 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="1" t="inlineStr">
+      <c r="A223" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('politics', 'right'))</t>
         </is>
@@ -7560,7 +7549,7 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="1" t="inlineStr">
+      <c r="A224" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('politics', 'left'))</t>
         </is>
@@ -7573,7 +7562,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="1" t="inlineStr">
+      <c r="A225" t="inlineStr">
         <is>
           <t>(('gender', 'non-binary'), ('politics', 'center'))</t>
         </is>
@@ -7586,7 +7575,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="1" t="inlineStr">
+      <c r="A226" t="inlineStr">
         <is>
           <t>(('gender', 'male'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7599,7 +7588,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="1" t="inlineStr">
+      <c r="A227" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7612,7 +7601,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="1" t="inlineStr">
+      <c r="A228" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7625,7 +7614,7 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="1" t="inlineStr">
+      <c r="A229" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'))</t>
         </is>
@@ -7638,7 +7627,7 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="1" t="inlineStr">
+      <c r="A230" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7651,7 +7640,7 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="1" t="inlineStr">
+      <c r="A231" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'), ('politics', 'center'))</t>
         </is>
@@ -7664,7 +7653,7 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="1" t="inlineStr">
+      <c r="A232" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7677,7 +7666,7 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="1" t="inlineStr">
+      <c r="A233" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('politics', 'center'))</t>
         </is>
@@ -7690,7 +7679,7 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="1" t="inlineStr">
+      <c r="A234" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -7703,7 +7692,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="1" t="inlineStr">
+      <c r="A235" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7716,7 +7705,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="1" t="inlineStr">
+      <c r="A236" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7729,7 +7718,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="1" t="inlineStr">
+      <c r="A237" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('politics', 'right'))</t>
         </is>
@@ -7742,7 +7731,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="1" t="inlineStr">
+      <c r="A238" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7755,7 +7744,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="1" t="inlineStr">
+      <c r="A239" t="inlineStr">
         <is>
           <t>(('education', 'low'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7768,7 +7757,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="1" t="inlineStr">
+      <c r="A240" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7781,7 +7770,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="1" t="inlineStr">
+      <c r="A241" t="inlineStr">
         <is>
           <t>(('gender', 'female'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7794,7 +7783,7 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="1" t="inlineStr">
+      <c r="A242" t="inlineStr">
         <is>
           <t>(('education', 'medium'), ('gender', 'non-binary'))</t>
         </is>
@@ -7807,7 +7796,7 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="1" t="inlineStr">
+      <c r="A243" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('gender', 'male'))</t>
         </is>
@@ -7820,7 +7809,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="1" t="inlineStr">
+      <c r="A244" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('gender', 'female'))</t>
         </is>
@@ -7833,7 +7822,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="1" t="inlineStr">
+      <c r="A245" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'low'), ('gender', 'non-binary'))</t>
         </is>
@@ -7846,7 +7835,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="1" t="inlineStr">
+      <c r="A246" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('politics', 'left'))</t>
         </is>
@@ -7859,7 +7848,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="1" t="inlineStr">
+      <c r="A247" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('politics', 'left'))</t>
         </is>
@@ -7872,7 +7861,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="1" t="inlineStr">
+      <c r="A248" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('orientation', 'heterosexual'))</t>
         </is>
@@ -7885,7 +7874,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="1" t="inlineStr">
+      <c r="A249" t="inlineStr">
         <is>
           <t>(('orientation', 'lgbtq+'), ('politics', 'right'))</t>
         </is>
@@ -7898,7 +7887,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="1" t="inlineStr">
+      <c r="A250" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('orientation', 'lgbtq+'))</t>
         </is>
@@ -7911,7 +7900,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="1" t="inlineStr">
+      <c r="A251" t="inlineStr">
         <is>
           <t>(('age', '25-50'), ('orientation', 'heterosexual'), ('politics', 'center'))</t>
         </is>
@@ -7924,7 +7913,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="1" t="inlineStr">
+      <c r="A252" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('politics', 'center'))</t>
         </is>
@@ -7937,7 +7926,7 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="1" t="inlineStr">
+      <c r="A253" t="inlineStr">
         <is>
           <t>(('education', 'high'), ('gender', 'female'), ('politics', 'left'))</t>
         </is>
@@ -7950,7 +7939,7 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="1" t="inlineStr">
+      <c r="A254" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('gender', 'female'))</t>
         </is>
@@ -7963,7 +7952,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="1" t="inlineStr">
+      <c r="A255" t="inlineStr">
         <is>
           <t>(('age', '&gt;50'), ('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -7976,7 +7965,7 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="1" t="inlineStr">
+      <c r="A256" t="inlineStr">
         <is>
           <t>(('age', '&lt;25'), ('education', 'medium'), ('politics', 'left'))</t>
         </is>
@@ -7986,6 +7975,99 @@
       </c>
       <c r="C256" t="n">
         <v>0.04614223257537056</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>retention_rate</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mean_leaves</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7.593023255813954</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mean_depth</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.316998468606432</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mean_residual_ndfu</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.1793278448401611</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mean_top_split_prg</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.4408721547050139</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>indeterminate_rate</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.006125574272588055</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dims_never_used</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>